<commit_message>
Cover profit-take and cash-reserve alerts in e2e fixture
</commit_message>
<xml_diff>
--- a/tests/fixtures/account_ikze_99999999_pl_xlsx_2024-12-31_2026-05-02.xlsx
+++ b/tests/fixtures/account_ikze_99999999_pl_xlsx_2024-12-31_2026-05-02.xlsx
@@ -1062,7 +1062,7 @@
     <outlinePr/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X16"/>
+  <dimension ref="B4:X16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.93359375" customWidth="1" style="49" min="1" max="1"/>
@@ -1131,12 +1131,12 @@
       <c r="D5" s="1" t="inlineStr"/>
       <c r="E5" s="1" t="inlineStr"/>
       <c r="F5" s="1" t="n"/>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="I5" s="11" t="inlineStr">
         <is>
           <t>99999999</t>
         </is>
       </c>
-      <c r="L5" s="6" t="n"/>
+      <c r="L5" s="11" t="n"/>
       <c r="O5" s="4" t="inlineStr"/>
       <c r="P5" s="4" t="inlineStr"/>
       <c r="Q5" s="4" t="inlineStr"/>
@@ -1185,13 +1185,13 @@
       <c r="F7" s="44" t="n">
         <v>4184.78</v>
       </c>
-      <c r="I7" s="6" t="n">
+      <c r="I7" s="11" t="n">
         <v>16755.21</v>
       </c>
-      <c r="L7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="6" t="n">
+      <c r="L7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="11" t="n">
         <v>4184.78</v>
       </c>
       <c r="R7" s="51" t="n">
@@ -1711,7 +1711,7 @@
     <outlinePr/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R19"/>
+  <dimension ref="B3:R19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.93359375" customWidth="1" style="49" min="1" max="1"/>
@@ -1772,12 +1772,12 @@
       <c r="D4" s="13" t="inlineStr"/>
       <c r="E4" s="13" t="inlineStr"/>
       <c r="F4" s="1" t="n"/>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>99999999</t>
         </is>
       </c>
-      <c r="L4" s="6" t="n"/>
+      <c r="L4" s="11" t="n"/>
       <c r="N4" s="15" t="inlineStr"/>
       <c r="O4" s="15" t="inlineStr"/>
       <c r="P4" s="15" t="inlineStr"/>
@@ -1820,16 +1820,16 @@
       <c r="D6" s="13" t="inlineStr"/>
       <c r="E6" s="13" t="inlineStr"/>
       <c r="F6" s="44" t="n">
-        <v>4184.78</v>
-      </c>
-      <c r="I6" s="6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I6" s="11" t="n">
         <v>16755.21</v>
       </c>
-      <c r="L6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="6" t="n">
-        <v>4184.78</v>
+      <c r="L6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="11" t="n">
+        <v>1000</v>
       </c>
       <c r="Q6" s="51" t="n">
         <v>0</v>
@@ -1974,7 +1974,7 @@
         <v>118.74</v>
       </c>
       <c r="H10" s="52" t="n">
-        <v>133.76</v>
+        <v>140</v>
       </c>
       <c r="I10" s="54" t="n">
         <v>1187.4</v>
@@ -1994,7 +1994,7 @@
         <v>0</v>
       </c>
       <c r="P10" s="56" t="n">
-        <v>150.2</v>
+        <v>212.6</v>
       </c>
       <c r="Q10" s="22" t="inlineStr"/>
     </row>
@@ -2452,7 +2452,7 @@
     <outlinePr/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="B3:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.93359375" customWidth="1" style="49" min="1" max="1"/>
@@ -2503,12 +2503,12 @@
       <c r="B4" s="13" t="inlineStr"/>
       <c r="C4" s="13" t="inlineStr"/>
       <c r="D4" s="1" t="n"/>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>99999999</t>
         </is>
       </c>
-      <c r="J4" s="6" t="n"/>
+      <c r="J4" s="11" t="n"/>
       <c r="L4" s="42" t="inlineStr"/>
       <c r="M4" s="42" t="inlineStr"/>
     </row>
@@ -2547,13 +2547,13 @@
       <c r="D6" s="44" t="n">
         <v>4184.78</v>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="G6" s="11" t="n">
         <v>16755.21</v>
       </c>
-      <c r="J6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="6" t="n">
+      <c r="J6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="11" t="n">
         <v>4184.78</v>
       </c>
       <c r="M6" s="51" t="n">
@@ -2717,7 +2717,7 @@
     <outlinePr/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="B3:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.93359375" customWidth="1" style="49" min="1" max="1"/>
@@ -2763,14 +2763,14 @@
       <c r="B4" s="13" t="inlineStr"/>
       <c r="C4" s="13" t="inlineStr"/>
       <c r="D4" s="1" t="n"/>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>99999999</t>
         </is>
       </c>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr"/>
+      <c r="F4" s="11" t="n"/>
+      <c r="G4" s="11" t="inlineStr"/>
+      <c r="H4" s="11" t="inlineStr"/>
     </row>
     <row r="5" ht="25.2" customHeight="1" s="49">
       <c r="B5" s="13" t="inlineStr"/>
@@ -2807,13 +2807,13 @@
       <c r="D6" s="44" t="n">
         <v>4184.78</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="11" t="n">
         <v>16755.21</v>
       </c>
-      <c r="F6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="6" t="n">
+      <c r="F6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="11" t="n">
         <v>4184.78</v>
       </c>
       <c r="H6" s="51" t="n">
@@ -2871,7 +2871,7 @@
           <t>Amount</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr"/>
+      <c r="H9" s="11" t="inlineStr"/>
     </row>
     <row r="10" ht="15.75" customHeight="1" s="49">
       <c r="B10" s="22" t="n">
@@ -2894,7 +2894,7 @@
       <c r="G10" s="56" t="n">
         <v>15611.4</v>
       </c>
-      <c r="H10" s="6" t="inlineStr"/>
+      <c r="H10" s="11" t="inlineStr"/>
     </row>
     <row r="11" ht="15.75" customHeight="1" s="49">
       <c r="B11" s="31" t="n">
@@ -2921,7 +2921,7 @@
       <c r="G11" s="64" t="n">
         <v>-2268</v>
       </c>
-      <c r="H11" s="6" t="inlineStr"/>
+      <c r="H11" s="11" t="inlineStr"/>
     </row>
     <row r="12" ht="15.75" customHeight="1" s="49">
       <c r="B12" s="22" t="n">
@@ -2948,7 +2948,7 @@
       <c r="G12" s="63" t="n">
         <v>-2336</v>
       </c>
-      <c r="H12" s="6" t="inlineStr"/>
+      <c r="H12" s="11" t="inlineStr"/>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="49">
       <c r="B13" s="31" t="n">
@@ -2975,7 +2975,7 @@
       <c r="G13" s="64" t="n">
         <v>-3696.34</v>
       </c>
-      <c r="H13" s="6" t="inlineStr"/>
+      <c r="H13" s="11" t="inlineStr"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="49">
       <c r="B14" s="22" t="n">
@@ -3002,7 +3002,7 @@
       <c r="G14" s="63" t="n">
         <v>-3717.31</v>
       </c>
-      <c r="H14" s="6" t="inlineStr"/>
+      <c r="H14" s="11" t="inlineStr"/>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="49">
       <c r="B15" s="31" t="n">
@@ -3025,7 +3025,7 @@
       <c r="G15" s="62" t="n">
         <v>11.01</v>
       </c>
-      <c r="H15" s="6" t="inlineStr"/>
+      <c r="H15" s="11" t="inlineStr"/>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="49">
       <c r="B16" s="22" t="n">
@@ -3052,7 +3052,7 @@
       <c r="G16" s="63" t="n">
         <v>-3445.34</v>
       </c>
-      <c r="H16" s="6" t="inlineStr"/>
+      <c r="H16" s="11" t="inlineStr"/>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="49">
       <c r="B17" s="31" t="n">
@@ -3079,7 +3079,7 @@
       <c r="G17" s="64" t="n">
         <v>-154</v>
       </c>
-      <c r="H17" s="6" t="inlineStr"/>
+      <c r="H17" s="11" t="inlineStr"/>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="49">
       <c r="B18" s="22" t="n">
@@ -3102,7 +3102,7 @@
       <c r="G18" s="56" t="n">
         <v>1.39</v>
       </c>
-      <c r="H18" s="6" t="inlineStr"/>
+      <c r="H18" s="11" t="inlineStr"/>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="49">
       <c r="B19" s="31" t="n">
@@ -3129,7 +3129,7 @@
       <c r="G19" s="62" t="n">
         <v>200.96</v>
       </c>
-      <c r="H19" s="6" t="inlineStr"/>
+      <c r="H19" s="11" t="inlineStr"/>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="49">
       <c r="B20" s="22" t="n">
@@ -3156,7 +3156,7 @@
       <c r="G20" s="56" t="n">
         <v>12.56</v>
       </c>
-      <c r="H20" s="6" t="inlineStr"/>
+      <c r="H20" s="11" t="inlineStr"/>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="49">
       <c r="B21" s="31" t="n">
@@ -3183,7 +3183,7 @@
       <c r="G21" s="62" t="n">
         <v>143.92</v>
       </c>
-      <c r="H21" s="6" t="inlineStr"/>
+      <c r="H21" s="11" t="inlineStr"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="49">
       <c r="B22" s="22" t="n">
@@ -3210,7 +3210,7 @@
       <c r="G22" s="56" t="n">
         <v>3445.34</v>
       </c>
-      <c r="H22" s="6" t="inlineStr"/>
+      <c r="H22" s="11" t="inlineStr"/>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="49">
       <c r="B23" s="31" t="n">
@@ -3237,7 +3237,7 @@
       <c r="G23" s="62" t="n">
         <v>156.45</v>
       </c>
-      <c r="H23" s="6" t="inlineStr"/>
+      <c r="H23" s="11" t="inlineStr"/>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="49">
       <c r="B24" s="22" t="n">
@@ -3264,7 +3264,7 @@
       <c r="G24" s="63" t="n">
         <v>-988.29</v>
       </c>
-      <c r="H24" s="6" t="inlineStr"/>
+      <c r="H24" s="11" t="inlineStr"/>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="49">
       <c r="B25" s="31" t="n">
@@ -3291,7 +3291,7 @@
       <c r="G25" s="64" t="n">
         <v>-11.68</v>
       </c>
-      <c r="H25" s="6" t="inlineStr"/>
+      <c r="H25" s="11" t="inlineStr"/>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="49">
       <c r="B26" s="22" t="n">
@@ -3318,7 +3318,7 @@
       <c r="G26" s="56" t="n">
         <v>541.25</v>
       </c>
-      <c r="H26" s="6" t="inlineStr"/>
+      <c r="H26" s="11" t="inlineStr"/>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="49">
       <c r="B27" s="31" t="n">
@@ -3345,7 +3345,7 @@
       <c r="G27" s="62" t="n">
         <v>3717.31</v>
       </c>
-      <c r="H27" s="6" t="inlineStr"/>
+      <c r="H27" s="11" t="inlineStr"/>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="49">
       <c r="B28" s="22" t="n">
@@ -3368,7 +3368,7 @@
       <c r="G28" s="56" t="n">
         <v>5.3</v>
       </c>
-      <c r="H28" s="6" t="inlineStr"/>
+      <c r="H28" s="11" t="inlineStr"/>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="49">
       <c r="B29" s="31" t="n">
@@ -3391,7 +3391,7 @@
       <c r="G29" s="62" t="n">
         <v>9.98</v>
       </c>
-      <c r="H29" s="6" t="inlineStr"/>
+      <c r="H29" s="11" t="inlineStr"/>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="49">
       <c r="B30" s="22" t="n">
@@ -3418,7 +3418,7 @@
       <c r="G30" s="63" t="n">
         <v>-1996</v>
       </c>
-      <c r="H30" s="6" t="inlineStr"/>
+      <c r="H30" s="11" t="inlineStr"/>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="49">
       <c r="B31" s="31" t="n">
@@ -3441,7 +3441,7 @@
       <c r="G31" s="62" t="n">
         <v>9.359999999999999</v>
       </c>
-      <c r="H31" s="6" t="inlineStr"/>
+      <c r="H31" s="11" t="inlineStr"/>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="49">
       <c r="B32" s="22" t="n">
@@ -3468,7 +3468,7 @@
       <c r="G32" s="63" t="n">
         <v>-49.56</v>
       </c>
-      <c r="H32" s="6" t="inlineStr"/>
+      <c r="H32" s="11" t="inlineStr"/>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="49">
       <c r="B33" s="31" t="n">
@@ -3495,7 +3495,7 @@
       <c r="G33" s="64" t="n">
         <v>-950.4</v>
       </c>
-      <c r="H33" s="6" t="inlineStr"/>
+      <c r="H33" s="11" t="inlineStr"/>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="49">
       <c r="B34" s="22" t="n">
@@ -3522,7 +3522,7 @@
       <c r="G34" s="63" t="n">
         <v>-154.17</v>
       </c>
-      <c r="H34" s="6" t="inlineStr"/>
+      <c r="H34" s="11" t="inlineStr"/>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="49">
       <c r="B35" s="31" t="n">
@@ -3549,7 +3549,7 @@
       <c r="G35" s="64" t="n">
         <v>-845.85</v>
       </c>
-      <c r="H35" s="6" t="inlineStr"/>
+      <c r="H35" s="11" t="inlineStr"/>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="49">
       <c r="B36" s="22" t="n">
@@ -3576,7 +3576,7 @@
       <c r="G36" s="63" t="n">
         <v>-147.42</v>
       </c>
-      <c r="H36" s="6" t="inlineStr"/>
+      <c r="H36" s="11" t="inlineStr"/>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="49">
       <c r="B37" s="31" t="n">
@@ -3603,7 +3603,7 @@
       <c r="G37" s="64" t="n">
         <v>-852.61</v>
       </c>
-      <c r="H37" s="6" t="inlineStr"/>
+      <c r="H37" s="11" t="inlineStr"/>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="49">
       <c r="B38" s="22" t="n">
@@ -3626,7 +3626,7 @@
       <c r="G38" s="56" t="n">
         <v>5.83</v>
       </c>
-      <c r="H38" s="6" t="inlineStr"/>
+      <c r="H38" s="11" t="inlineStr"/>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="49">
       <c r="B39" s="31" t="n">
@@ -3653,7 +3653,7 @@
       <c r="G39" s="64" t="n">
         <v>-163.2</v>
       </c>
-      <c r="H39" s="6" t="inlineStr"/>
+      <c r="H39" s="11" t="inlineStr"/>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="49">
       <c r="B40" s="22" t="n">
@@ -3680,7 +3680,7 @@
       <c r="G40" s="56" t="n">
         <v>1996</v>
       </c>
-      <c r="H40" s="6" t="inlineStr"/>
+      <c r="H40" s="11" t="inlineStr"/>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="49">
       <c r="B41" s="31" t="n">
@@ -3707,7 +3707,7 @@
       <c r="G41" s="64" t="n">
         <v>-2.1</v>
       </c>
-      <c r="H41" s="6" t="inlineStr"/>
+      <c r="H41" s="11" t="inlineStr"/>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="49">
       <c r="B42" s="22" t="n">
@@ -3734,7 +3734,7 @@
       <c r="G42" s="56" t="n">
         <v>2268</v>
       </c>
-      <c r="H42" s="6" t="inlineStr"/>
+      <c r="H42" s="11" t="inlineStr"/>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="49">
       <c r="B43" s="31" t="n">
@@ -3757,7 +3757,7 @@
       <c r="G43" s="62" t="n">
         <v>3.36</v>
       </c>
-      <c r="H43" s="6" t="inlineStr"/>
+      <c r="H43" s="11" t="inlineStr"/>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="49">
       <c r="B44" s="22" t="n">
@@ -3784,7 +3784,7 @@
       <c r="G44" s="63" t="n">
         <v>-1187.4</v>
       </c>
-      <c r="H44" s="6" t="inlineStr"/>
+      <c r="H44" s="11" t="inlineStr"/>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="49">
       <c r="B45" s="31" t="n">
@@ -3807,7 +3807,7 @@
       <c r="G45" s="62" t="n">
         <v>6.11</v>
       </c>
-      <c r="H45" s="6" t="inlineStr"/>
+      <c r="H45" s="11" t="inlineStr"/>
     </row>
     <row r="46" ht="15.75" customHeight="1" s="49">
       <c r="B46" s="22" t="n">
@@ -3834,7 +3834,7 @@
       <c r="G46" s="63" t="n">
         <v>-47.98</v>
       </c>
-      <c r="H46" s="6" t="inlineStr"/>
+      <c r="H46" s="11" t="inlineStr"/>
     </row>
     <row r="47" ht="15.75" customHeight="1" s="49">
       <c r="B47" s="31" t="n">
@@ -3861,7 +3861,7 @@
       <c r="G47" s="64" t="n">
         <v>-952</v>
       </c>
-      <c r="H47" s="6" t="inlineStr"/>
+      <c r="H47" s="11" t="inlineStr"/>
     </row>
     <row r="48" ht="17" customHeight="1" s="49">
       <c r="B48" s="39" t="inlineStr">

</xml_diff>